<commit_message>
updated excel file added new sheet
</commit_message>
<xml_diff>
--- a/test file.xlsx
+++ b/test file.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="9000" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="test file" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1251,4 +1252,51 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>